<commit_message>
Cambios menores (solo para poder cambiar de branch)
</commit_message>
<xml_diff>
--- a/data/france/p4_modeling/2024-10-03/df_best_model.xlsx
+++ b/data/france/p4_modeling/2024-10-03/df_best_model.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,22 +674,22 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>1152</v>
+        <v>1520</v>
       </c>
       <c r="B4" t="n">
-        <v>11.67794357665307</v>
+        <v>10.62859635869195</v>
       </c>
       <c r="C4" t="n">
-        <v>94.63268692064449</v>
+        <v>80.66617535706892</v>
       </c>
       <c r="D4" t="n">
-        <v>5149.405535813347</v>
+        <v>5340.054891020053</v>
       </c>
       <c r="E4" t="n">
-        <v>40.22973074854178</v>
+        <v>41.71917883609417</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>(128, 23)</t>
+          <t>(128, 19)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>2.444932790133563</v>
+        <v>2.925182350346448</v>
       </c>
       <c r="N4" t="n">
         <v>55</v>
@@ -728,43 +728,43 @@
         <v>42</v>
       </c>
       <c r="Q4" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="R4" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="S4" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="T4" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="U4" t="n">
-        <v>59.375</v>
+        <v>57.03125</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>412</v>
+        <v>1152</v>
       </c>
       <c r="B5" t="n">
-        <v>13.31279969417804</v>
+        <v>11.67794357665307</v>
       </c>
       <c r="C5" t="n">
-        <v>16.80344963956195</v>
+        <v>94.63268692064449</v>
       </c>
       <c r="D5" t="n">
-        <v>4119.76841186301</v>
+        <v>5149.405535813347</v>
       </c>
       <c r="E5" t="n">
-        <v>32.18569071767976</v>
+        <v>40.22973074854178</v>
       </c>
       <c r="F5" t="n">
         <v>-0.25</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>kelly</t>
+          <t>linear</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -774,11 +774,11 @@
         <v>0</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>(128, 22)</t>
+          <t>(128, 23)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>1.417650040340893</v>
+        <v>2.444932790133563</v>
       </c>
       <c r="N5" t="n">
         <v>55</v>
@@ -799,13 +799,13 @@
         <v>42</v>
       </c>
       <c r="Q5" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="R5" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="S5" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="T5" t="n">
         <v>76</v>
@@ -816,26 +816,26 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>548</v>
+        <v>412</v>
       </c>
       <c r="B6" t="n">
-        <v>10.65158161462233</v>
+        <v>13.31279969417804</v>
       </c>
       <c r="C6" t="n">
-        <v>29.89100187240196</v>
+        <v>16.80344963956195</v>
       </c>
       <c r="D6" t="n">
-        <v>3612.94840523903</v>
+        <v>4119.76841186301</v>
       </c>
       <c r="E6" t="n">
-        <v>28.22615941592992</v>
+        <v>32.18569071767976</v>
       </c>
       <c r="F6" t="n">
         <v>-0.25</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>linear</t>
+          <t>kelly</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -845,11 +845,11 @@
         <v>0</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>(128, 45)</t>
+          <t>(128, 22)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>1.649950067244612</v>
+        <v>1.417650040340893</v>
       </c>
       <c r="N6" t="n">
         <v>55</v>
@@ -870,43 +870,43 @@
         <v>42</v>
       </c>
       <c r="Q6" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="R6" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S6" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="T6" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="U6" t="n">
-        <v>60.15625</v>
+        <v>59.375</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>188</v>
+        <v>844</v>
       </c>
       <c r="B7" t="n">
-        <v>2.6881063188868</v>
+        <v>17.14439398793253</v>
       </c>
       <c r="C7" t="n">
-        <v>4.837825201751883</v>
+        <v>11.40613794902004</v>
       </c>
       <c r="D7" t="n">
-        <v>2436.694779932905</v>
+        <v>3857.49506608566</v>
       </c>
       <c r="E7" t="n">
-        <v>19.03667796822582</v>
+        <v>30.13668020379422</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>linear</t>
+          <t>kelly</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -916,11 +916,11 @@
         <v>0</v>
       </c>
       <c r="J7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>(128, 27)</t>
+          <t>(128, 23)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>6.081817350181781</v>
+        <v>0.7578154249725364</v>
       </c>
       <c r="N7" t="n">
         <v>55</v>
@@ -941,36 +941,36 @@
         <v>42</v>
       </c>
       <c r="Q7" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="R7" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="S7" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="T7" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="U7" t="n">
-        <v>58.59375</v>
+        <v>59.375</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>494</v>
+        <v>548</v>
       </c>
       <c r="B8" t="n">
-        <v>6.247812577820886</v>
+        <v>10.65158161462233</v>
       </c>
       <c r="C8" t="n">
-        <v>4.865616162725917</v>
+        <v>29.89100187240196</v>
       </c>
       <c r="D8" t="n">
-        <v>1365.404274636484</v>
+        <v>3612.94840523903</v>
       </c>
       <c r="E8" t="n">
-        <v>10.66722089559753</v>
+        <v>28.22615941592992</v>
       </c>
       <c r="F8" t="n">
         <v>-0.25</v>
@@ -991,7 +991,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>(128, 9)</t>
+          <t>(128, 45)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>0.7073528955502131</v>
+        <v>1.649950067244612</v>
       </c>
       <c r="N8" t="n">
         <v>55</v>
@@ -1012,39 +1012,39 @@
         <v>42</v>
       </c>
       <c r="Q8" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="R8" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="S8" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="T8" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="U8" t="n">
-        <v>57.03125</v>
+        <v>60.15625</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>192</v>
+        <v>928</v>
       </c>
       <c r="B9" t="n">
-        <v>6.597803576580078</v>
+        <v>20.91221511571387</v>
       </c>
       <c r="C9" t="n">
-        <v>6.020805146830856</v>
+        <v>18.25846929320853</v>
       </c>
       <c r="D9" t="n">
-        <v>1140.98776591331</v>
+        <v>3081.461688751634</v>
       </c>
       <c r="E9" t="n">
-        <v>8.913966921197737</v>
+        <v>24.07391944337214</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>(128, 14)</t>
+          <t>(128, 7)</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>0.351050666746012</v>
+        <v>0.1511893556069295</v>
       </c>
       <c r="N9" t="n">
         <v>55</v>
@@ -1086,33 +1086,33 @@
         <v>53</v>
       </c>
       <c r="R9" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="S9" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="T9" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U9" t="n">
-        <v>57.8125</v>
+        <v>58.59375</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>1248</v>
+        <v>188</v>
       </c>
       <c r="B10" t="n">
-        <v>6.191467732992717</v>
+        <v>2.6881063188868</v>
       </c>
       <c r="C10" t="n">
-        <v>12.7923581728683</v>
+        <v>4.837825201751883</v>
       </c>
       <c r="D10" t="n">
-        <v>1095.73644462219</v>
+        <v>2436.694779932905</v>
       </c>
       <c r="E10" t="n">
-        <v>8.560440973610858</v>
+        <v>19.03667796822582</v>
       </c>
       <c r="F10" t="n">
         <v>-0.5</v>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>(128, 16)</t>
+          <t>(128, 27)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>0.3826190077668499</v>
+        <v>6.081817350181781</v>
       </c>
       <c r="N10" t="n">
         <v>55</v>
@@ -1154,10 +1154,10 @@
         <v>42</v>
       </c>
       <c r="Q10" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="R10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S10" t="n">
         <v>43</v>
@@ -1171,19 +1171,19 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>409</v>
+        <v>747</v>
       </c>
       <c r="B11" t="n">
-        <v>5.154703703649305</v>
+        <v>6.615652295182992</v>
       </c>
       <c r="C11" t="n">
-        <v>18.89785077063781</v>
+        <v>7.885489745511215</v>
       </c>
       <c r="D11" t="n">
-        <v>1047.497831779373</v>
+        <v>1701.102044230671</v>
       </c>
       <c r="E11" t="n">
-        <v>8.183576810776355</v>
+        <v>13.28985972055212</v>
       </c>
       <c r="F11" t="n">
         <v>-0.5</v>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>(128, 22)</t>
+          <t>(128, 38)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>0.5875940269821407</v>
+        <v>1.008850998748645</v>
       </c>
       <c r="N11" t="n">
         <v>55</v>
@@ -1225,57 +1225,57 @@
         <v>42</v>
       </c>
       <c r="Q11" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="R11" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="S11" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="T11" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="U11" t="n">
-        <v>57.8125</v>
+        <v>59.375</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>798</v>
+        <v>1064</v>
       </c>
       <c r="B12" t="n">
-        <v>1.717436250610635</v>
+        <v>3.160110772109764</v>
       </c>
       <c r="C12" t="n">
-        <v>2.076354332628146</v>
+        <v>5.617198468338315</v>
       </c>
       <c r="D12" t="n">
-        <v>913.6071106070494</v>
+        <v>1600.059748756923</v>
       </c>
       <c r="E12" t="n">
-        <v>7.137555551617574</v>
+        <v>12.50046678716346</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>linear</t>
+          <t>kelly</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>(128, 11)</t>
+          <t>(128, 46)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>3.15593623872782</v>
+        <v>2.955705254856574</v>
       </c>
       <c r="N12" t="n">
         <v>55</v>
@@ -1296,39 +1296,39 @@
         <v>42</v>
       </c>
       <c r="Q12" t="n">
+        <v>54</v>
+      </c>
+      <c r="R12" t="n">
+        <v>22</v>
+      </c>
+      <c r="S12" t="n">
         <v>52</v>
       </c>
-      <c r="R12" t="n">
-        <v>29</v>
-      </c>
-      <c r="S12" t="n">
-        <v>47</v>
-      </c>
       <c r="T12" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U12" t="n">
-        <v>57.8125</v>
+        <v>57.03125</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>542</v>
+        <v>494</v>
       </c>
       <c r="B13" t="n">
-        <v>3.144377583146938</v>
+        <v>6.247812577820886</v>
       </c>
       <c r="C13" t="n">
-        <v>5.261930900629505</v>
+        <v>4.865616162725917</v>
       </c>
       <c r="D13" t="n">
-        <v>895.8100657347202</v>
+        <v>1365.404274636484</v>
       </c>
       <c r="E13" t="n">
-        <v>6.998516138552501</v>
+        <v>10.66722089559753</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>(128, 8)</t>
+          <t>(128, 9)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>1.225723836750002</v>
+        <v>0.7073528955502131</v>
       </c>
       <c r="N13" t="n">
         <v>55</v>
@@ -1367,13 +1367,13 @@
         <v>42</v>
       </c>
       <c r="Q13" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="R13" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="S13" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="T13" t="n">
         <v>73</v>
@@ -1384,22 +1384,22 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>892</v>
+        <v>682</v>
       </c>
       <c r="B14" t="n">
-        <v>3.737448248548367</v>
+        <v>-0.1553024802942338</v>
       </c>
       <c r="C14" t="n">
-        <v>14.78405065737587</v>
+        <v>4.082174581906375</v>
       </c>
       <c r="D14" t="n">
-        <v>591.6988494562331</v>
+        <v>1146.345374560551</v>
       </c>
       <c r="E14" t="n">
-        <v>4.622647261376821</v>
+        <v>8.955823238754302</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.25</v>
+        <v>-0.5</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>(128, 24)</t>
+          <t>(128, 29)</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>0.2368458247340997</v>
+        <v>58.66696849777757</v>
       </c>
       <c r="N14" t="n">
         <v>55</v>
@@ -1438,13 +1438,13 @@
         <v>42</v>
       </c>
       <c r="Q14" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="R14" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="S14" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="T14" t="n">
         <v>72</v>
@@ -1455,40 +1455,40 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>456</v>
+        <v>192</v>
       </c>
       <c r="B15" t="n">
-        <v>2.747417875372478</v>
+        <v>6.597803576580078</v>
       </c>
       <c r="C15" t="n">
-        <v>5.809805336691072</v>
+        <v>6.020805146830856</v>
       </c>
       <c r="D15" t="n">
-        <v>466.5777057566661</v>
+        <v>1140.98776591331</v>
       </c>
       <c r="E15" t="n">
-        <v>3.645138326223954</v>
+        <v>8.913966921197737</v>
       </c>
       <c r="F15" t="n">
         <v>-0.5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>kelly</t>
+          <t>linear</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>(128, 35)</t>
+          <t>(128, 14)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>0.3267506042304425</v>
+        <v>0.351050666746012</v>
       </c>
       <c r="N15" t="n">
         <v>55</v>
@@ -1509,13 +1509,13 @@
         <v>42</v>
       </c>
       <c r="Q15" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="R15" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="S15" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="T15" t="n">
         <v>74</v>
@@ -1526,19 +1526,19 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>1406</v>
+        <v>1248</v>
       </c>
       <c r="B16" t="n">
-        <v>3.320497050649384</v>
+        <v>6.191467732992717</v>
       </c>
       <c r="C16" t="n">
-        <v>1.7576954399556</v>
+        <v>12.7923581728683</v>
       </c>
       <c r="D16" t="n">
-        <v>459.9703320633252</v>
+        <v>1095.73644462219</v>
       </c>
       <c r="E16" t="n">
-        <v>3.593518219244728</v>
+        <v>8.560440973610858</v>
       </c>
       <c r="F16" t="n">
         <v>-0.5</v>
@@ -1549,7 +1549,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>(128, 13)</t>
+          <t>(128, 16)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>0.082222981809892</v>
+        <v>0.3826190077668499</v>
       </c>
       <c r="N16" t="n">
         <v>55</v>
@@ -1580,36 +1580,36 @@
         <v>42</v>
       </c>
       <c r="Q16" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="R16" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="S16" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="T16" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="U16" t="n">
-        <v>56.25</v>
+        <v>58.59375</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>734</v>
+        <v>409</v>
       </c>
       <c r="B17" t="n">
-        <v>2.842523239822908</v>
+        <v>5.154703703649305</v>
       </c>
       <c r="C17" t="n">
-        <v>1.048033895763465</v>
+        <v>18.89785077063781</v>
       </c>
       <c r="D17" t="n">
-        <v>388.7440827593852</v>
+        <v>1047.497831779373</v>
       </c>
       <c r="E17" t="n">
-        <v>3.037063146557697</v>
+        <v>8.183576810776355</v>
       </c>
       <c r="F17" t="n">
         <v>-0.5</v>
@@ -1620,7 +1620,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>(128, 15)</t>
+          <t>(128, 22)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>0.06843916137934859</v>
+        <v>0.5875940269821407</v>
       </c>
       <c r="N17" t="n">
         <v>55</v>
@@ -1651,57 +1651,57 @@
         <v>42</v>
       </c>
       <c r="Q17" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="R17" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="S17" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="T17" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="U17" t="n">
-        <v>55.46875</v>
+        <v>57.8125</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>190</v>
+        <v>798</v>
       </c>
       <c r="B18" t="n">
-        <v>2.527602982721143</v>
+        <v>1.717436250610635</v>
       </c>
       <c r="C18" t="n">
-        <v>6.535841372708513</v>
+        <v>2.076354332628146</v>
       </c>
       <c r="D18" t="n">
-        <v>377.5646026020904</v>
+        <v>913.6071106070494</v>
       </c>
       <c r="E18" t="n">
-        <v>2.949723457828831</v>
+        <v>7.137555551617574</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>kelly</t>
+          <t>linear</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>(128, 14)</t>
+          <t>(128, 11)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1710,7 +1710,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>0.1670042637207388</v>
+        <v>3.15593623872782</v>
       </c>
       <c r="N18" t="n">
         <v>55</v>
@@ -1722,36 +1722,36 @@
         <v>42</v>
       </c>
       <c r="Q18" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R18" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="S18" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="T18" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="U18" t="n">
-        <v>55.46875</v>
+        <v>57.8125</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B19" t="n">
-        <v>2.287688715792938</v>
+        <v>3.144377583146938</v>
       </c>
       <c r="C19" t="n">
-        <v>5.184245034245201</v>
+        <v>5.261930900629505</v>
       </c>
       <c r="D19" t="n">
-        <v>347.9138998354917</v>
+        <v>895.8100657347202</v>
       </c>
       <c r="E19" t="n">
-        <v>2.718077342464779</v>
+        <v>6.998516138552501</v>
       </c>
       <c r="F19" t="n">
         <v>-0.5</v>
@@ -1762,50 +1762,1257 @@
         </is>
       </c>
       <c r="H19" t="n">
+        <v>40</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>(128, 8)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>1.225723836750002</v>
+      </c>
+      <c r="N19" t="n">
+        <v>55</v>
+      </c>
+      <c r="O19" t="n">
+        <v>31</v>
+      </c>
+      <c r="P19" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>56</v>
+      </c>
+      <c r="R19" t="n">
+        <v>29</v>
+      </c>
+      <c r="S19" t="n">
+        <v>43</v>
+      </c>
+      <c r="T19" t="n">
+        <v>73</v>
+      </c>
+      <c r="U19" t="n">
+        <v>57.03125</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>1302</v>
+      </c>
+      <c r="B20" t="n">
+        <v>5.494494109650239</v>
+      </c>
+      <c r="C20" t="n">
+        <v>19.52983959836838</v>
+      </c>
+      <c r="D20" t="n">
+        <v>868.4296369090864</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.784606538352238</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>40</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>(128, 24)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0.2348009485415798</v>
+      </c>
+      <c r="N20" t="n">
+        <v>55</v>
+      </c>
+      <c r="O20" t="n">
+        <v>31</v>
+      </c>
+      <c r="P20" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>58</v>
+      </c>
+      <c r="R20" t="n">
+        <v>37</v>
+      </c>
+      <c r="S20" t="n">
+        <v>33</v>
+      </c>
+      <c r="T20" t="n">
+        <v>72</v>
+      </c>
+      <c r="U20" t="n">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>1072</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-0.1564422124073559</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.0519702749208578</v>
+      </c>
+      <c r="D21" t="n">
+        <v>846.4803457950156</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6.61312770152356</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>40</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>(128, 16)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>43.27201597164712</v>
+      </c>
+      <c r="N21" t="n">
+        <v>55</v>
+      </c>
+      <c r="O21" t="n">
+        <v>31</v>
+      </c>
+      <c r="P21" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>57</v>
+      </c>
+      <c r="R21" t="n">
+        <v>23</v>
+      </c>
+      <c r="S21" t="n">
+        <v>48</v>
+      </c>
+      <c r="T21" t="n">
+        <v>75</v>
+      </c>
+      <c r="U21" t="n">
+        <v>58.59375</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>270</v>
+      </c>
+      <c r="B22" t="n">
+        <v>2.431725371042962</v>
+      </c>
+      <c r="C22" t="n">
+        <v>11.42411915822972</v>
+      </c>
+      <c r="D22" t="n">
+        <v>750.9358450657816</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5.866686289576418</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>30</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>(128, 20)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>1.412561204253179</v>
+      </c>
+      <c r="N22" t="n">
+        <v>55</v>
+      </c>
+      <c r="O22" t="n">
+        <v>31</v>
+      </c>
+      <c r="P22" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>64</v>
+      </c>
+      <c r="R22" t="n">
+        <v>21</v>
+      </c>
+      <c r="S22" t="n">
+        <v>43</v>
+      </c>
+      <c r="T22" t="n">
+        <v>74</v>
+      </c>
+      <c r="U22" t="n">
+        <v>57.8125</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>1134</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1.755557572027648</v>
+      </c>
+      <c r="C23" t="n">
+        <v>5.246412455151308</v>
+      </c>
+      <c r="D23" t="n">
+        <v>626.0025564887748</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4.890644972568553</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>30</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="b">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>(128, 20)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>1.785807227569254</v>
+      </c>
+      <c r="N23" t="n">
+        <v>55</v>
+      </c>
+      <c r="O23" t="n">
+        <v>31</v>
+      </c>
+      <c r="P23" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>48</v>
+      </c>
+      <c r="R23" t="n">
+        <v>28</v>
+      </c>
+      <c r="S23" t="n">
+        <v>52</v>
+      </c>
+      <c r="T23" t="n">
+        <v>71</v>
+      </c>
+      <c r="U23" t="n">
+        <v>55.46875</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>892</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3.737448248548367</v>
+      </c>
+      <c r="C24" t="n">
+        <v>14.78405065737587</v>
+      </c>
+      <c r="D24" t="n">
+        <v>591.6988494562331</v>
+      </c>
+      <c r="E24" t="n">
+        <v>4.622647261376821</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="b">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>(128, 24)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>0.2368458247340997</v>
+      </c>
+      <c r="N24" t="n">
+        <v>55</v>
+      </c>
+      <c r="O24" t="n">
+        <v>31</v>
+      </c>
+      <c r="P24" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>54</v>
+      </c>
+      <c r="R24" t="n">
+        <v>28</v>
+      </c>
+      <c r="S24" t="n">
+        <v>46</v>
+      </c>
+      <c r="T24" t="n">
+        <v>72</v>
+      </c>
+      <c r="U24" t="n">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>686</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1.706999050039278</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.256915801675563</v>
+      </c>
+      <c r="D25" t="n">
+        <v>518.6216950986992</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4.051731992958588</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>30</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>(128, 15)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>1.373599442170374</v>
+      </c>
+      <c r="N25" t="n">
+        <v>55</v>
+      </c>
+      <c r="O25" t="n">
+        <v>31</v>
+      </c>
+      <c r="P25" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>53</v>
+      </c>
+      <c r="R25" t="n">
+        <v>24</v>
+      </c>
+      <c r="S25" t="n">
+        <v>51</v>
+      </c>
+      <c r="T25" t="n">
+        <v>72</v>
+      </c>
+      <c r="U25" t="n">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>387</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2.817234077924213</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4.255959822753518</v>
+      </c>
+      <c r="D26" t="n">
+        <v>518.3080863519374</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4.049281924624511</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>kelly</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>(128, 31)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>0.4373253384781191</v>
+      </c>
+      <c r="N26" t="n">
+        <v>55</v>
+      </c>
+      <c r="O26" t="n">
+        <v>31</v>
+      </c>
+      <c r="P26" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>59</v>
+      </c>
+      <c r="R26" t="n">
+        <v>23</v>
+      </c>
+      <c r="S26" t="n">
+        <v>46</v>
+      </c>
+      <c r="T26" t="n">
+        <v>75</v>
+      </c>
+      <c r="U26" t="n">
+        <v>58.59375</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>456</v>
+      </c>
+      <c r="B27" t="n">
+        <v>2.747417875372478</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5.809805336691072</v>
+      </c>
+      <c r="D27" t="n">
+        <v>466.5777057566661</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.645138326223954</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>kelly</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>30</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>(128, 35)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>0.3267506042304425</v>
+      </c>
+      <c r="N27" t="n">
+        <v>55</v>
+      </c>
+      <c r="O27" t="n">
+        <v>31</v>
+      </c>
+      <c r="P27" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>59</v>
+      </c>
+      <c r="R27" t="n">
+        <v>27</v>
+      </c>
+      <c r="S27" t="n">
+        <v>42</v>
+      </c>
+      <c r="T27" t="n">
+        <v>74</v>
+      </c>
+      <c r="U27" t="n">
+        <v>57.8125</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>1406</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3.320497050649384</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.7576954399556</v>
+      </c>
+      <c r="D28" t="n">
+        <v>459.9703320633252</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3.593518219244728</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>30</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>(128, 13)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>0.082222981809892</v>
+      </c>
+      <c r="N28" t="n">
+        <v>55</v>
+      </c>
+      <c r="O28" t="n">
+        <v>31</v>
+      </c>
+      <c r="P28" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>50</v>
+      </c>
+      <c r="R28" t="n">
+        <v>29</v>
+      </c>
+      <c r="S28" t="n">
+        <v>49</v>
+      </c>
+      <c r="T28" t="n">
+        <v>72</v>
+      </c>
+      <c r="U28" t="n">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>1283</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2.630083324262056</v>
+      </c>
+      <c r="C29" t="n">
+        <v>7.995611447992042</v>
+      </c>
+      <c r="D29" t="n">
+        <v>438.8527011972963</v>
+      </c>
+      <c r="E29" t="n">
+        <v>3.428536728103877</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>30</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>(128, 61)</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>0.30358483188583</v>
+      </c>
+      <c r="N29" t="n">
+        <v>55</v>
+      </c>
+      <c r="O29" t="n">
+        <v>31</v>
+      </c>
+      <c r="P29" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>72</v>
+      </c>
+      <c r="R29" t="n">
+        <v>21</v>
+      </c>
+      <c r="S29" t="n">
+        <v>35</v>
+      </c>
+      <c r="T29" t="n">
+        <v>73</v>
+      </c>
+      <c r="U29" t="n">
+        <v>57.03125</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="B30" t="n">
+        <v>1.971495760331153</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3.422450607542578</v>
+      </c>
+      <c r="D30" t="n">
+        <v>435.1174494848775</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3.399355074100605</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>30</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>(128, 17)</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>0.7242517800442108</v>
+      </c>
+      <c r="N30" t="n">
+        <v>55</v>
+      </c>
+      <c r="O30" t="n">
+        <v>31</v>
+      </c>
+      <c r="P30" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>46</v>
+      </c>
+      <c r="R30" t="n">
+        <v>28</v>
+      </c>
+      <c r="S30" t="n">
+        <v>54</v>
+      </c>
+      <c r="T30" t="n">
+        <v>71</v>
+      </c>
+      <c r="U30" t="n">
+        <v>55.46875</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B31" t="n">
+        <v>1.302423229407821</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1.417453600313426</v>
+      </c>
+      <c r="D31" t="n">
+        <v>427.4625529258519</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3.339551194733218</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="b">
+        <v>0</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>(128, 60)</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>1.564105982854458</v>
+      </c>
+      <c r="N31" t="n">
+        <v>55</v>
+      </c>
+      <c r="O31" t="n">
+        <v>31</v>
+      </c>
+      <c r="P31" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>51</v>
+      </c>
+      <c r="R31" t="n">
+        <v>24</v>
+      </c>
+      <c r="S31" t="n">
+        <v>53</v>
+      </c>
+      <c r="T31" t="n">
+        <v>70</v>
+      </c>
+      <c r="U31" t="n">
+        <v>54.6875</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>734</v>
+      </c>
+      <c r="B32" t="n">
+        <v>2.842523239822908</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1.048033895763465</v>
+      </c>
+      <c r="D32" t="n">
+        <v>388.7440827593852</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3.037063146557697</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>30</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="b">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>(128, 15)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>0.06843916137934859</v>
+      </c>
+      <c r="N32" t="n">
+        <v>55</v>
+      </c>
+      <c r="O32" t="n">
+        <v>31</v>
+      </c>
+      <c r="P32" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>56</v>
+      </c>
+      <c r="R32" t="n">
+        <v>30</v>
+      </c>
+      <c r="S32" t="n">
+        <v>42</v>
+      </c>
+      <c r="T32" t="n">
+        <v>71</v>
+      </c>
+      <c r="U32" t="n">
+        <v>55.46875</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>190</v>
+      </c>
+      <c r="B33" t="n">
+        <v>2.527602982721143</v>
+      </c>
+      <c r="C33" t="n">
+        <v>6.535841372708513</v>
+      </c>
+      <c r="D33" t="n">
+        <v>377.5646026020904</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.949723457828831</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>kelly</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>20</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>(128, 14)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>0.1670042637207388</v>
+      </c>
+      <c r="N33" t="n">
+        <v>55</v>
+      </c>
+      <c r="O33" t="n">
+        <v>31</v>
+      </c>
+      <c r="P33" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>51</v>
+      </c>
+      <c r="R33" t="n">
+        <v>34</v>
+      </c>
+      <c r="S33" t="n">
+        <v>43</v>
+      </c>
+      <c r="T33" t="n">
+        <v>71</v>
+      </c>
+      <c r="U33" t="n">
+        <v>55.46875</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>533</v>
+      </c>
+      <c r="B34" t="n">
+        <v>-0.462070663055101</v>
+      </c>
+      <c r="C34" t="n">
+        <v>7.32201553052399</v>
+      </c>
+      <c r="D34" t="n">
+        <v>355.6074643752623</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2.778183315431737</v>
+      </c>
+      <c r="F34" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
         <v>25</v>
       </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="b">
-        <v>0</v>
-      </c>
-      <c r="K19" t="inlineStr">
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>(128, 22)</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>7.012464191219264</v>
+      </c>
+      <c r="N34" t="n">
+        <v>55</v>
+      </c>
+      <c r="O34" t="n">
+        <v>31</v>
+      </c>
+      <c r="P34" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>70</v>
+      </c>
+      <c r="R34" t="n">
+        <v>26</v>
+      </c>
+      <c r="S34" t="n">
+        <v>32</v>
+      </c>
+      <c r="T34" t="n">
+        <v>71</v>
+      </c>
+      <c r="U34" t="n">
+        <v>55.46875</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>538</v>
+      </c>
+      <c r="B35" t="n">
+        <v>2.287688715792938</v>
+      </c>
+      <c r="C35" t="n">
+        <v>5.184245034245201</v>
+      </c>
+      <c r="D35" t="n">
+        <v>347.9138998354917</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.718077342464779</v>
+      </c>
+      <c r="F35" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="b">
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>(128, 15)</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>neural_networ</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
         <v>0.1881325128286361</v>
       </c>
-      <c r="N19" t="n">
-        <v>55</v>
-      </c>
-      <c r="O19" t="n">
-        <v>31</v>
-      </c>
-      <c r="P19" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q19" t="n">
+      <c r="N35" t="n">
+        <v>55</v>
+      </c>
+      <c r="O35" t="n">
+        <v>31</v>
+      </c>
+      <c r="P35" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q35" t="n">
         <v>51</v>
       </c>
-      <c r="R19" t="n">
+      <c r="R35" t="n">
         <v>30</v>
       </c>
-      <c r="S19" t="n">
+      <c r="S35" t="n">
         <v>47</v>
       </c>
-      <c r="T19" t="n">
+      <c r="T35" t="n">
         <v>71</v>
       </c>
-      <c r="U19" t="n">
+      <c r="U35" t="n">
         <v>55.46875</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>1278</v>
+      </c>
+      <c r="B36" t="n">
+        <v>1.885650296152705</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.3750404575517217</v>
+      </c>
+      <c r="D36" t="n">
+        <v>311.098367968475</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2.430455999753711</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>30</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>(128, 12)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>neural_networ</t>
+        </is>
+      </c>
+      <c r="M36" t="n">
+        <v>0.2889219197815067</v>
+      </c>
+      <c r="N36" t="n">
+        <v>55</v>
+      </c>
+      <c r="O36" t="n">
+        <v>31</v>
+      </c>
+      <c r="P36" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>53</v>
+      </c>
+      <c r="R36" t="n">
+        <v>39</v>
+      </c>
+      <c r="S36" t="n">
+        <v>36</v>
+      </c>
+      <c r="T36" t="n">
+        <v>68</v>
+      </c>
+      <c r="U36" t="n">
+        <v>53.125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>